<commit_message>
Restore STEP-TOD direct observation gate source cells
</commit_message>
<xml_diff>
--- a/NewLogic 03.05.2026/ST_Target_Observed_Environment_Diagnostic.xlsx
+++ b/NewLogic 03.05.2026/ST_Target_Observed_Environment_Diagnostic.xlsx
@@ -5804,7 +5804,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -6174,7 +6174,11 @@
       <c r="R7" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S7" s="31"/>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T7" s="31"/>
       <c r="U7" s="31"/>
       <c r="V7" s="31"/>
@@ -6235,7 +6239,11 @@
       <c r="R8" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S8" s="31"/>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T8" s="31"/>
       <c r="U8" s="31"/>
       <c r="V8" s="31"/>
@@ -6296,7 +6304,11 @@
       <c r="R9" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S9" s="31"/>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T9" s="31"/>
       <c r="U9" s="31"/>
       <c r="V9" s="31"/>
@@ -6357,7 +6369,11 @@
       <c r="R10" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S10" s="31"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T10" s="31"/>
       <c r="U10" s="31"/>
       <c r="V10" s="31"/>
@@ -6418,7 +6434,11 @@
       <c r="R11" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S11" s="31"/>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T11" s="31"/>
       <c r="U11" s="31"/>
       <c r="V11" s="31"/>
@@ -6479,7 +6499,11 @@
       <c r="R12" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S12" s="31"/>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T12" s="31"/>
       <c r="U12" s="31"/>
       <c r="V12" s="31"/>
@@ -6540,7 +6564,11 @@
       <c r="R13" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S13" s="31"/>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T13" s="31"/>
       <c r="U13" s="31"/>
       <c r="V13" s="31"/>
@@ -6601,7 +6629,11 @@
       <c r="R14" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S14" s="31"/>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T14" s="31"/>
       <c r="U14" s="31"/>
       <c r="V14" s="31"/>
@@ -6662,7 +6694,11 @@
       <c r="R15" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S15" s="31"/>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T15" s="31"/>
       <c r="U15" s="31"/>
       <c r="V15" s="31"/>
@@ -6723,7 +6759,11 @@
       <c r="R16" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S16" s="31"/>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T16" s="31"/>
       <c r="U16" s="31"/>
       <c r="V16" s="31"/>
@@ -6784,7 +6824,11 @@
       <c r="R17" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S17" s="31"/>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T17" s="31"/>
       <c r="U17" s="31"/>
       <c r="V17" s="31"/>
@@ -6845,7 +6889,11 @@
       <c r="R18" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S18" s="31"/>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T18" s="31"/>
       <c r="U18" s="31"/>
       <c r="V18" s="31"/>
@@ -6906,7 +6954,11 @@
       <c r="R19" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S19" s="31"/>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T19" s="31"/>
       <c r="U19" s="31"/>
       <c r="V19" s="31"/>
@@ -6967,7 +7019,11 @@
       <c r="R20" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S20" s="31"/>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T20" s="31"/>
       <c r="U20" s="31"/>
       <c r="V20" s="31"/>
@@ -7028,7 +7084,11 @@
       <c r="R21" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S21" s="31"/>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T21" s="31"/>
       <c r="U21" s="31"/>
       <c r="V21" s="31"/>
@@ -7089,7 +7149,11 @@
       <c r="R22" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S22" s="31"/>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T22" s="31"/>
       <c r="U22" s="31"/>
       <c r="V22" s="31"/>
@@ -7150,7 +7214,11 @@
       <c r="R23" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S23" s="31"/>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T23" s="31"/>
       <c r="U23" s="31"/>
       <c r="V23" s="31"/>
@@ -7211,7 +7279,11 @@
       <c r="R24" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="S24" s="31"/>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T24" s="31"/>
       <c r="U24" s="31"/>
       <c r="V24" s="31"/>
@@ -7272,7 +7344,11 @@
       <c r="R25" s="18" t="s">
         <v>210</v>
       </c>
-      <c r="S25" s="34"/>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Direct Observation Gate (v3.1) — Did your diligence team produce direct, observable evidence on this dimension?</t>
+        </is>
+      </c>
       <c r="T25" s="34"/>
       <c r="U25" s="34"/>
       <c r="V25" s="34"/>

</xml_diff>